<commit_message>
experimento registrado + carga bien env
</commit_message>
<xml_diff>
--- a/runs/experiments.xlsx
+++ b/runs/experiments.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -737,6 +737,57 @@
         <v>45677</v>
       </c>
       <c r="O6" t="inlineStr">
+        <is>
+          <t>subiendo batch size</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>/Feb16_14_10_20</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>42</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>64</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H7" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1480.782152093256</v>
+      </c>
+      <c r="N7" t="n">
+        <v>57803</v>
+      </c>
+      <c r="O7" t="inlineStr">
         <is>
           <t>subiendo batch size</t>
         </is>

</xml_diff>

<commit_message>
cambios para q funcione
</commit_message>
<xml_diff>
--- a/runs/experiments.xlsx
+++ b/runs/experiments.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -788,6 +788,57 @@
         <v>57803</v>
       </c>
       <c r="O7" t="inlineStr">
+        <is>
+          <t>subiendo batch size</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>/Feb19_20_16_59</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>42</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="D8" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E8" t="n">
+        <v>64</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H8" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I8" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="M8" t="n">
+        <v>346.6151197853893</v>
+      </c>
+      <c r="N8" t="n">
+        <v>61750</v>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>subiendo batch size</t>
         </is>

</xml_diff>

<commit_message>
wrapper reward y rangos termination
</commit_message>
<xml_diff>
--- a/runs/experiments.xlsx
+++ b/runs/experiments.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -890,6 +890,57 @@
         <v>465868</v>
       </c>
       <c r="O9" t="inlineStr">
+        <is>
+          <t>subiendo batch size</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>/Feb23_17_42_17</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>42</v>
+      </c>
+      <c r="C10" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D10" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>64</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I10" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="M10" t="n">
+        <v>107.4727475967969</v>
+      </c>
+      <c r="N10" t="n">
+        <v>96740</v>
+      </c>
+      <c r="O10" t="inlineStr">
         <is>
           <t>subiendo batch size</t>
         </is>

</xml_diff>

<commit_message>
codigo tal cual para el entrenamiento de Feb26_10_30_09
</commit_message>
<xml_diff>
--- a/runs/experiments.xlsx
+++ b/runs/experiments.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -997,6 +997,57 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>/Feb24_20_17_56</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>42</v>
+      </c>
+      <c r="C12" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E12" t="n">
+        <v>64</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H12" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="M12" t="n">
+        <v>852.0568986491583</v>
+      </c>
+      <c r="N12" t="n">
+        <v>106008</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>subiendo batch size</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
rainbow funcionando primer try
</commit_message>
<xml_diff>
--- a/runs/experiments.xlsx
+++ b/runs/experiments.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -1048,6 +1048,77 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Feb28_18_41_08</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>42</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Rainbow(C51+Double+PER+Nstep+Noisy+Dueling)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F13" t="n">
+        <v>64</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="J13" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K13" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>51</v>
+      </c>
+      <c r="P13" t="n">
+        <v>-50</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>200</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="S13" t="n">
+        <v>777.0320642574716</v>
+      </c>
+      <c r="T13" t="n">
+        <v>28703</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>rainbow C51 training script</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ficheros rainbow last update
</commit_message>
<xml_diff>
--- a/runs/experiments.xlsx
+++ b/runs/experiments.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -1119,6 +1119,148 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Mar05_18_29_34</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>42</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Rainbow(C51+Double+PER+Nstep+Noisy+Dueling)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="E14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F14" t="n">
+        <v>64</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="J14" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K14" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>51</v>
+      </c>
+      <c r="P14" t="n">
+        <v>-50</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="S14" t="n">
+        <v>948.3970224506344</v>
+      </c>
+      <c r="T14" t="n">
+        <v>30742</v>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>rainbow C51 training script</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mar09_11_49_29</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>42</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Rainbow(C51+Double+PER+Nstep+Noisy+Dueling)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="E15" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F15" t="n">
+        <v>64</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="J15" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K15" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>51</v>
+      </c>
+      <c r="P15" t="n">
+        <v>-80</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>500</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="S15" t="n">
+        <v>2048.3372077319</v>
+      </c>
+      <c r="T15" t="n">
+        <v>30069</v>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>rainbow C51 training script</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ablation 1 y 2
</commit_message>
<xml_diff>
--- a/runs/experiments.xlsx
+++ b/runs/experiments.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -1261,6 +1261,130 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mar11_00_23_57_ablation1_nodistributional</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>42</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Rainbow ablation 1 (NO Distributional RL; keep Double+PER+Nstep+Noisy+Dueling)</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F16" t="n">
+        <v>64</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="J16" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K16" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1334.434560013533</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>33320</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>ablation study part 1: Rainbow without C51/distributional component</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mar12_18_29_22</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>42</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Rainbow ablation 2 (WITH Distributional RL, WITHOUT PER)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="E17" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F17" t="n">
+        <v>64</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="J17" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K17" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L17" t="n">
+        <v>51</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-80</v>
+      </c>
+      <c r="N17" t="n">
+        <v>500</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1574.804011108224</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>31939</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>ablation study part 2: Rainbow keeps C51/Double/Dueling/Noisy/n-step and removes PER</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>